<commit_message>
more fresh off Claude changes
</commit_message>
<xml_diff>
--- a/RotorSizingResults.xlsx
+++ b/RotorSizingResults.xlsx
@@ -433,7 +433,7 @@
   <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="105" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,177 +446,177 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PROVISIONAL RESULTS for the 8-lap force-based load case (Regenerative_Braking_Forces_8_Laps.csv).</t>
+          <t>CORRECTED RESULTS for the 8-lap force-based load case (Regenerative_Braking_Forces_8_Laps.csv).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated from a verified port of RotorSizingOptimizer.m (cross-checked against GNU Octave and an</t>
+          <t>This replaces the previous RotorSizingResults.xlsx, which used two bugs now fixed:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>independent Python port), not from MATLAB itself. Re-running RotorSizingOptimizer.m overwrites this file.</t>
+          <t xml:space="preserve">  1. A variable-name bug (velx instead of CYC.velx) that only affected the Euler-stability warning,</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     not the physics.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER INPUTS USED HERE (results are conditional on them):</t>
+          <t xml:space="preserve">  2. A real physics bug: the Speed_mps column is mislabeled and is actually in MPH. It was being</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tbias_front = 0.60     -- REQUIRED, not yet supplied (now splits FrictionBrakeForce_N directly)</t>
+          <t xml:space="preserve">     used as-is, AND the m/s-calibrated velx_threshold (34 m/s) was then zeroing out 53% of the rows</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  T_target_F  = 800      -- REQUIRED, not yet supplied</t>
+          <t xml:space="preserve">     (every row where true speed exceeded 34 "m/s", i.e. most of the file, since mph values run</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     much higher than m/s ones). That dropped over half the drive cycle from the friction-energy</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>WHAT CHANGED THIS SESSION:</t>
+          <t xml:space="preserve">     calculation, understating front/rear friction heat by roughly 10x. Confirmed the mph hypothesis</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1. Friction heat is now a DIRECT measurement: |FrictionBrakeForce_N| x distance, split by</t>
+          <t xml:space="preserve">     independently via the wheel-radius check: converting mph-&gt;m/s gives an implied wheel radius of</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Tbias_front and 0.5 L/R, because FrictionBrakeForce_N is confirmed to be the actual</t>
+          <t xml:space="preserve">     0.203 m vs WheelR = 0.213 m (-4.7%), the same sign and magnitude of mismatch found on the prior</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     longitudinal friction force at the contact patch (already net of regen). This replaces the</t>
+          <t xml:space="preserve">     (correctly-labeled) MotorTorque.csv load case. Fixed by converting Speed_mps x 0.44704 before</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     old KE-loss/regen-subtraction estimate and removes the max(...,0) clamp entirely - there is</t>
+          <t xml:space="preserve">     any other use.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     nothing left to clamp, and the rear-corner LOWER BOUND caveat from the last load case no</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     longer applies.</t>
+          <t>Generated from a verified port of RotorSizingOptimizer.m (cross-checked against GNU Octave and an</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. Braking-active gate is now RequiredBrakingMagnitude_N &gt; 0 (a direct force column), not an</t>
+          <t>independent Python port), not from MATLAB itself. Re-running RotorSizingOptimizer.m overwrites this file.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     inferred pedal-force-and-deceleration heuristic.</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Verified identities on the corrected columns: FrictionBrakeForce_N + AppliedRegenForce_N =</t>
+          <t>PLACEHOLDER INPUTS USED HERE (results are conditional on them):</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     -RequiredBrakingMagnitude_N (max err 1.0e-6 N); LongitudinalForce_N = -RequiredBrakingMagnitude_N</t>
+          <t xml:space="preserve">  Tbias_front = 0.60     -- REQUIRED, not yet supplied</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     - AeroDragMagnitude_N on every braking row (max err 5.0e-7 N).</t>
+          <t xml:space="preserve">  T_target_F  = 800      -- REQUIRED, not yet supplied</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  4. regen_front_frac_a/b is no longer used by the heat calculation for this format (kept in the</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     parameter sheet only for the legacy torque-based format).</t>
+          <t>RESULT ON THIS LOAD CASE (corrected): both rotors still sit on the geometric mass floor (t_min,</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>phi_max) - that part is unaffected by the speed-unit bug, since it is set by geometry alone. But the</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>RESULT ON THIS LOAD CASE: both rotors sit on the geometric mass floor (t_min, phi_max) regardless</t>
+          <t>required area and resulting temperatures are now materially higher: front A_target = 0.004527 m^2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>of T_target - the 8-lap cycle is thermally trivial (peak 112.9 degF front / 99.8 degF rear at the</t>
+          <t>(was 0.0 m^2), peak 350.1 degF at the existence-proof geometry (was 112.9 degF); rear A_target =</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>proof geometry) because AvailableRegenMagnitude_N covers most of RequiredBrakingMagnitude_N on this</t>
+          <t>0.001855 m^2 (was 0.0 m^2), peak 253.4 degF (was 99.8 degF). T_target is still fully slack at 800 degF</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>run. Sensitivity to h_w and T_target is flat for the same reason (mass floor governs).</t>
+          <t>- the mass floor still governs - but the margin is far smaller than previously reported.</t>
         </is>
       </c>
     </row>
@@ -626,14 +626,14 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>The existence-proof geometry demonstrates that a buildable (t, Ar, L) exists at m_target.</t>
+          <t>The existence-proof geometry demonstrates that a buildable (t, Ar, L) exists at m_target and clears</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>It is NOT the recommended design - that is what the generative-design tool is for.</t>
+          <t>A_target with margin. It is NOT the recommended design - that is what the generative-design tool is for.</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
         <v>0.114293</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0</v>
+        <v>0.00452709</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.01508293</v>
@@ -866,19 +866,19 @@
         <v>0.114293</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>112.88</v>
+        <v>350.13</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>99.98</v>
+        <v>320.53</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>98.59999999999999</v>
+        <v>257.36</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>112.88</v>
+        <v>350.13</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>273.04</v>
+        <v>800</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>0.114293</v>
@@ -893,7 +893,7 @@
         <v>0.4834</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>0.00079</v>
+        <v>0.00071</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>0.123664</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0</v>
+        <v>0.00185519</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>0.01586979</v>
@@ -944,19 +944,19 @@
         <v>0.123664</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>99.81999999999999</v>
+        <v>253.44</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>91.89</v>
+        <v>234.24</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>90.34</v>
+        <v>191.37</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>99.81999999999999</v>
+        <v>253.44</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>200.49</v>
+        <v>800</v>
       </c>
       <c r="S3" s="2" t="n">
         <v>0.123664</v>
@@ -971,7 +971,7 @@
         <v>0.5266</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>0.00082</v>
+        <v>0.00073</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
         <v>0.114293</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>0.00452709</v>
       </c>
     </row>
     <row r="3">
@@ -1054,7 +1054,7 @@
         <v>0.114293</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>0.005659</v>
       </c>
     </row>
     <row r="4">
@@ -1072,7 +1072,7 @@
         <v>0.114293</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>0.003773</v>
       </c>
     </row>
     <row r="5">
@@ -1090,7 +1090,7 @@
         <v>0.114293</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>0.00487</v>
       </c>
     </row>
     <row r="6">
@@ -1108,7 +1108,7 @@
         <v>0.114293</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>0.004204</v>
       </c>
     </row>
     <row r="7">
@@ -1126,7 +1126,7 @@
         <v>0.123664</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>0.00185519</v>
       </c>
     </row>
     <row r="8">
@@ -1144,7 +1144,7 @@
         <v>0.123664</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>0.002319</v>
       </c>
     </row>
     <row r="9">
@@ -1162,7 +1162,7 @@
         <v>0.123664</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>0.001546</v>
       </c>
     </row>
     <row r="10">
@@ -1180,7 +1180,7 @@
         <v>0.123664</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>0.002123</v>
       </c>
     </row>
     <row r="11">
@@ -1198,7 +1198,7 @@
         <v>0.123664</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>0.001599</v>
       </c>
     </row>
   </sheetData>

</xml_diff>